<commit_message>
Convolution and Combined Models not working. Else ok
</commit_message>
<xml_diff>
--- a/Datos Problemas no ideales.xlsx
+++ b/Datos Problemas no ideales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\TFG Base Isabela Fons\ReactorApp toolbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E406E97-7175-44EF-9684-2844923FAA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C455A9-A60C-49B1-996C-8DA87F18A2E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34785" yWindow="4830" windowWidth="15825" windowHeight="10500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="2340" windowWidth="15825" windowHeight="10500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -376,10 +376,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
         <v>0</v>
@@ -402,10 +402,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -428,10 +428,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -454,10 +454,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="D6">
         <v>15</v>
@@ -506,10 +506,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>77</v>
       </c>
       <c r="D7">
         <v>20</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <v>70</v>
       </c>
       <c r="D8">
         <v>30</v>
@@ -558,10 +558,10 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="D9">
         <v>40</v>
@@ -584,10 +584,10 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="D10">
         <v>50</v>
@@ -610,10 +610,10 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="B11">
-        <v>2.2000000000000002</v>
+        <v>32</v>
       </c>
       <c r="D11">
         <v>70</v>
@@ -636,10 +636,10 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B12">
-        <v>1.5</v>
+        <v>15</v>
       </c>
       <c r="D12">
         <v>100</v>
@@ -662,10 +662,10 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B13">
-        <v>0.6</v>
+        <v>7</v>
       </c>
       <c r="D13">
         <v>125</v>
@@ -688,10 +688,10 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D14">
         <v>150</v>

</xml_diff>

<commit_message>
Gran cambio a cinética modular
</commit_message>
<xml_diff>
--- a/Datos Problemas no ideales.xlsx
+++ b/Datos Problemas no ideales.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\TFG Base Isabela Fons\ReactorApp toolbox\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\ReactorApp toolbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F143DB1B-E937-4040-A479-777569EDE438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70D6994-F092-49BB-B3A9-151E697AD48B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30180" yWindow="2700" windowWidth="15825" windowHeight="10500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Giro en el cambio de unidades
</commit_message>
<xml_diff>
--- a/Datos Problemas no ideales.xlsx
+++ b/Datos Problemas no ideales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\ReactorApp toolbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1123FD9-E97D-46BB-8B5F-DD34687E8D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AEBEC2-5AA0-4250-9C62-4B564C2E131A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5310" yWindow="2325" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -365,10 +365,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -395,8 +395,10 @@
       <c r="L1" s="2">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>_xlfn.XLOOKUP($D$2,$1:$1,3:3,"no",0,1)</f>
         <v>0</v>
@@ -428,8 +430,10 @@
       <c r="L2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A14" si="0">_xlfn.XLOOKUP($D$2,$1:$1,4:4,"no",0,1)</f>
         <v>5</v>
@@ -457,7 +461,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -485,7 +489,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -513,7 +517,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -541,7 +545,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -569,7 +573,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -597,7 +601,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -625,7 +629,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>70</v>
@@ -653,7 +657,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>100</v>
@@ -681,7 +685,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>125</v>
@@ -709,7 +713,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>150</v>
@@ -737,7 +741,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>175</v>
@@ -765,7 +769,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <f>IF(_xlfn.XLOOKUP($D$2,$1:$1,16:16,"no",0,1)=0,"",_xlfn.XLOOKUP($D$2,$1:$1,16:16,"no",0,1))</f>
         <v>200</v>
@@ -793,7 +797,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E16">
         <v>200</v>
       </c>

</xml_diff>

<commit_message>
rework UI Prediction Models
</commit_message>
<xml_diff>
--- a/Datos Problemas no ideales.xlsx
+++ b/Datos Problemas no ideales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\ReactorApp toolbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF920CA-E133-4337-86DF-BCABE1D7AB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED29E05-C129-42A5-BA80-81B0B7561476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -440,11 +440,11 @@
     <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A14" si="0">_xlfn.XLOOKUP($D$3,$1:$1,3:3,"no",0,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2">
         <f t="shared" ref="B2:B14" si="1">_xlfn.XLOOKUP($D$3,$1:$1,3:3,"no",0,-1)</f>
-        <v>9</v>
+        <v>112</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>2</v>
@@ -480,14 +480,14 @@
     <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <f t="shared" si="1"/>
-        <v>35</v>
+        <v>95.8</v>
       </c>
       <c r="D3" s="3">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -517,11 +517,11 @@
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <f t="shared" si="1"/>
-        <v>52</v>
+        <v>82.2</v>
       </c>
       <c r="F4">
         <v>5</v>
@@ -552,11 +552,11 @@
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B5">
         <f t="shared" si="1"/>
-        <v>65</v>
+        <v>70.599999999999994</v>
       </c>
       <c r="F5">
         <v>10</v>
@@ -587,11 +587,11 @@
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B6">
         <f t="shared" si="1"/>
-        <v>82</v>
+        <v>60.9</v>
       </c>
       <c r="F6">
         <v>15</v>
@@ -622,11 +622,11 @@
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B7">
         <f t="shared" si="1"/>
-        <v>77</v>
+        <v>45.6</v>
       </c>
       <c r="F7">
         <v>20</v>
@@ -657,11 +657,11 @@
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="B8">
         <f t="shared" si="1"/>
-        <v>70</v>
+        <v>34.5</v>
       </c>
       <c r="F8">
         <v>30</v>
@@ -692,11 +692,11 @@
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B9">
         <f t="shared" si="1"/>
-        <v>56</v>
+        <v>26.3</v>
       </c>
       <c r="F9">
         <v>40</v>
@@ -727,11 +727,11 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="B10">
         <f t="shared" si="1"/>
-        <v>47</v>
+        <v>15.7</v>
       </c>
       <c r="F10">
         <v>50</v>
@@ -762,11 +762,11 @@
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B11">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>7.67</v>
       </c>
       <c r="F11">
         <v>70</v>
@@ -797,11 +797,11 @@
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>125</v>
       </c>
       <c r="B12">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>5.1100000000000003</v>
       </c>
       <c r="F12">
         <v>100</v>
@@ -832,11 +832,11 @@
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>41</v>
+        <v>150</v>
       </c>
       <c r="B13">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="F13">
         <v>125</v>
@@ -867,11 +867,11 @@
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>52</v>
+        <v>175</v>
       </c>
       <c r="B14">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>1.73</v>
       </c>
       <c r="F14">
         <v>150</v>
@@ -900,13 +900,13 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" t="str">
+      <c r="A15">
         <f t="shared" ref="A15:A20" si="3">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1))</f>
-        <v/>
-      </c>
-      <c r="B15" t="str">
+        <v>200</v>
+      </c>
+      <c r="B15">
         <f t="shared" ref="B15:B20" si="4">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1))</f>
-        <v/>
+        <v>0.9</v>
       </c>
       <c r="F15">
         <v>175</v>

</xml_diff>

<commit_message>
New UI TAB 1 & 2
</commit_message>
<xml_diff>
--- a/Datos Problemas no ideales.xlsx
+++ b/Datos Problemas no ideales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\ReactorApp toolbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED29E05-C129-42A5-BA80-81B0B7561476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A7D0043-0100-4CE0-AE37-389189B9BA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -440,11 +440,11 @@
     <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A14" si="0">_xlfn.XLOOKUP($D$3,$1:$1,3:3,"no",0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <f t="shared" ref="B2:B14" si="1">_xlfn.XLOOKUP($D$3,$1:$1,3:3,"no",0,-1)</f>
-        <v>112</v>
+        <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>2</v>
@@ -480,14 +480,14 @@
     <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <f t="shared" si="1"/>
-        <v>95.8</v>
+        <v>35</v>
       </c>
       <c r="D3" s="3">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -517,11 +517,11 @@
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <f t="shared" si="1"/>
-        <v>82.2</v>
+        <v>52</v>
       </c>
       <c r="F4">
         <v>5</v>
@@ -552,11 +552,11 @@
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <f t="shared" si="1"/>
-        <v>70.599999999999994</v>
+        <v>65</v>
       </c>
       <c r="F5">
         <v>10</v>
@@ -587,11 +587,11 @@
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <f t="shared" si="1"/>
-        <v>60.9</v>
+        <v>82</v>
       </c>
       <c r="F6">
         <v>15</v>
@@ -622,11 +622,11 @@
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <f t="shared" si="1"/>
-        <v>45.6</v>
+        <v>77</v>
       </c>
       <c r="F7">
         <v>20</v>
@@ -657,11 +657,11 @@
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <f t="shared" si="1"/>
-        <v>34.5</v>
+        <v>70</v>
       </c>
       <c r="F8">
         <v>30</v>
@@ -692,11 +692,11 @@
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B9">
         <f t="shared" si="1"/>
-        <v>26.3</v>
+        <v>56</v>
       </c>
       <c r="F9">
         <v>40</v>
@@ -727,11 +727,11 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <f t="shared" si="1"/>
-        <v>15.7</v>
+        <v>47</v>
       </c>
       <c r="F10">
         <v>50</v>
@@ -762,11 +762,11 @@
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="B11">
         <f t="shared" si="1"/>
-        <v>7.67</v>
+        <v>32</v>
       </c>
       <c r="F11">
         <v>70</v>
@@ -797,11 +797,11 @@
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="B12">
         <f t="shared" si="1"/>
-        <v>5.1100000000000003</v>
+        <v>15</v>
       </c>
       <c r="F12">
         <v>100</v>
@@ -832,11 +832,11 @@
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>41</v>
       </c>
       <c r="B13">
         <f t="shared" si="1"/>
-        <v>2.5499999999999998</v>
+        <v>7</v>
       </c>
       <c r="F13">
         <v>125</v>
@@ -867,11 +867,11 @@
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>175</v>
+        <v>52</v>
       </c>
       <c r="B14">
         <f t="shared" si="1"/>
-        <v>1.73</v>
+        <v>3</v>
       </c>
       <c r="F14">
         <v>150</v>
@@ -900,13 +900,13 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="A15" t="str">
         <f t="shared" ref="A15:A20" si="3">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1))</f>
-        <v>200</v>
-      </c>
-      <c r="B15">
+        <v/>
+      </c>
+      <c r="B15" t="str">
         <f t="shared" ref="B15:B20" si="4">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1))</f>
-        <v>0.9</v>
+        <v/>
       </c>
       <c r="F15">
         <v>175</v>

</xml_diff>